<commit_message>
Ajout d'un script pour automatiser l'installation de Proxmox VE
</commit_message>
<xml_diff>
--- a/data/vm-cfg.xlsx
+++ b/data/vm-cfg.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
   <si>
     <t>VMName</t>
   </si>
@@ -37,10 +37,13 @@
     <t>Hyper-V</t>
   </si>
   <si>
+    <t>Proxmox VE</t>
+  </si>
+  <si>
+    <t>Serveur AD + DS + DNS</t>
+  </si>
+  <si>
     <t>Proxmox</t>
-  </si>
-  <si>
-    <t>Serveur AD + DS + DNS</t>
   </si>
   <si>
     <t>Serveur Nextcloud</t>
@@ -329,12 +332,12 @@
         <v>40</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" s="5">
         <v>2</v>
@@ -346,12 +349,12 @@
         <v>24</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B6" s="5">
         <v>2</v>
@@ -363,12 +366,12 @@
         <v>16</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="5">
         <v>2</v>
@@ -380,12 +383,12 @@
         <v>40</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B8" s="5">
         <v>2</v>
@@ -397,12 +400,12 @@
         <v>40</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B10" s="5">
         <f>SUM(B2:B3)</f>
@@ -423,7 +426,7 @@
     </row>
     <row r="11">
       <c r="A11" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="5">

</xml_diff>